<commit_message>
feat: Refactorizar exportación de licencias y actualizar tabla de certificados
</commit_message>
<xml_diff>
--- a/app/Templates/template_exportar_datos_licencias.xlsx
+++ b/app/Templates/template_exportar_datos_licencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dacuna\Herd\itse-app\app\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CDCE17C-3455-437B-952B-4442A6772D9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D122DB4-54FC-48C3-9922-1706E9D7D435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C21146A1-4A55-4D73-B125-4AB76F93B3DF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>ITEM</t>
   </si>
@@ -69,6 +69,18 @@
   </si>
   <si>
     <t>Reporte Certificados de Licencia de Funcionamiento</t>
+  </si>
+  <si>
+    <t>RUC</t>
+  </si>
+  <si>
+    <t>DIRECCION</t>
+  </si>
+  <si>
+    <t>ZONIFICACION</t>
+  </si>
+  <si>
+    <t>RESOLUCION</t>
   </si>
 </sst>
 </file>
@@ -162,11 +174,12 @@
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -174,9 +187,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -568,98 +584,111 @@
     <col min="2" max="2" width="7.5703125" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="45.5703125" style="10" customWidth="1"/>
+    <col min="5" max="5" width="45.5703125" style="5" customWidth="1"/>
     <col min="6" max="6" width="60.42578125" customWidth="1"/>
     <col min="7" max="7" width="57.5703125" customWidth="1"/>
     <col min="8" max="8" width="23" customWidth="1"/>
     <col min="9" max="9" width="40.140625" customWidth="1"/>
     <col min="10" max="10" width="45.5703125" customWidth="1"/>
     <col min="11" max="11" width="45.140625" customWidth="1"/>
+    <col min="12" max="13" width="31.85546875" customWidth="1"/>
     <col min="15" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
     </row>
     <row r="2" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="6"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="O6" s="4"/>
-      <c r="P6" s="4"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="2" t="s">
         <v>1</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="K7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="L7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="M7" s="10" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: se añadio un filtro multiple para giros
</commit_message>
<xml_diff>
--- a/app/Templates/template_exportar_datos_licencias.xlsx
+++ b/app/Templates/template_exportar_datos_licencias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jpolo\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53AEF4CD-909A-40ED-845C-C346CEFCFFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CF83C4F-FC55-44F9-8F58-B2850D991C0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C21146A1-4A55-4D73-B125-4AB76F93B3DF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>ITEM</t>
   </si>
@@ -84,6 +84,9 @@
   </si>
   <si>
     <t>FECHA EMISION</t>
+  </si>
+  <si>
+    <t>GIROS</t>
   </si>
 </sst>
 </file>
@@ -592,10 +595,10 @@
     <col min="8" max="8" width="23" customWidth="1"/>
     <col min="9" max="9" width="40.140625" customWidth="1"/>
     <col min="10" max="10" width="45.5703125" customWidth="1"/>
-    <col min="11" max="11" width="45.140625" customWidth="1"/>
+    <col min="11" max="11" width="61.7109375" customWidth="1"/>
     <col min="12" max="13" width="31.85546875" customWidth="1"/>
     <col min="14" max="14" width="32.140625" customWidth="1"/>
-    <col min="15" max="15" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.7109375" customWidth="1"/>
     <col min="16" max="16" width="13.140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -692,15 +695,18 @@
         <v>6</v>
       </c>
       <c r="K7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="L7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="M7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="M7" s="7" t="s">
+      <c r="N7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="N7" s="7" t="s">
+      <c r="O7" s="7" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>